<commit_message>
Actualización de homogeneización, bases e inputs para la construcción de tablas
</commit_message>
<xml_diff>
--- a/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
+++ b/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAURA\Trabajo\EAFIT\Proyectos\Provincias\git\Proyecto-Provincias\01_Data\00_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD65A1C-483A-4B7D-80DB-F29834ABF1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40848687-80D0-4615-BF9D-1322E3409D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{87AE0CA6-2098-4AEE-924F-4FDC71F02AC8}"/>
   </bookViews>
@@ -28,13 +28,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Diccionario_Base!$A$1:$I$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Distribución homogeneización'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Indicadores adicionales'!$A$1:$C$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Indicadores clave'!$A$1:$W$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Indicadores clave'!$A$1:$W$222</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inventario variables'!$A$1:$Q$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Variables nuevas (propuesta)'!$A$1:$J$2</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="2" r:id="rId10"/>
+    <pivotCache cacheId="0" r:id="rId10"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8862" uniqueCount="1293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8875" uniqueCount="1300">
   <si>
     <t>Tipo</t>
   </si>
@@ -4060,6 +4060,27 @@
   </si>
   <si>
     <t>Sí está en la base de datos, pero no consigo la información</t>
+  </si>
+  <si>
+    <t>tasa_mortalidad</t>
+  </si>
+  <si>
+    <t>2005-2024</t>
+  </si>
+  <si>
+    <t>DATOS SALUD.xlsx, hoja "tasa de mortalidad general"</t>
+  </si>
+  <si>
+    <t>Mortalidad general 2024.xlsx</t>
+  </si>
+  <si>
+    <t>Se actualizó DATOS SALUD.xlsx, hoja "tasa de mortalidad general" fuente: https://dssa.gov.co/OSSSA/Mortalidad.html</t>
+  </si>
+  <si>
+    <t>DATOS SALUD.xlsx (hoja: tasa de mortalidad general)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tasa de mortalidad general por cada cien mil habitantes </t>
   </si>
 </sst>
 </file>
@@ -4232,7 +4253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -4368,9 +4389,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -8554,7 +8572,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B14FD70E-783B-46DF-ACED-476E396A4C66}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B14FD70E-783B-46DF-ACED-476E396A4C66}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B81" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField showAll="0"/>
@@ -32769,8 +32787,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:W221"/>
+  <dimension ref="A1:W222"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" style="6" bestFit="1" customWidth="1"/>
@@ -33108,7 +33125,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" ht="30" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>124</v>
       </c>
@@ -33164,7 +33181,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="7" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>424</v>
       </c>
@@ -33220,7 +33237,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>426</v>
       </c>
@@ -33276,7 +33293,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>443</v>
       </c>
@@ -33333,7 +33350,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="79.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="79.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>457</v>
       </c>
@@ -33437,7 +33454,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>220</v>
       </c>
@@ -33481,7 +33498,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>220</v>
       </c>
@@ -33517,7 +33534,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>112</v>
       </c>
@@ -33570,7 +33587,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="23.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>220</v>
       </c>
@@ -33614,7 +33631,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="42.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>220</v>
       </c>
@@ -33658,7 +33675,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="31.8" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" ht="31.8" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="33" t="s">
         <v>116</v>
       </c>
@@ -33976,7 +33993,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" ht="30" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>220</v>
       </c>
@@ -34009,7 +34026,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="45" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="45" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>220</v>
       </c>
@@ -34225,7 +34242,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="29" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" s="33" t="s">
         <v>76</v>
       </c>
@@ -34271,7 +34288,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" s="33" t="s">
         <v>80</v>
       </c>
@@ -34317,7 +34334,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="31" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" s="33" t="s">
         <v>82</v>
       </c>
@@ -34363,7 +34380,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="32" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" s="33" t="s">
         <v>84</v>
       </c>
@@ -34409,7 +34426,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="33" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>218</v>
       </c>
@@ -34682,7 +34699,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" s="33" t="s">
         <v>508</v>
       </c>
@@ -34727,7 +34744,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
         <v>510</v>
       </c>
@@ -34772,7 +34789,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="33" t="s">
         <v>512</v>
       </c>
@@ -34817,7 +34834,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="33" t="s">
         <v>514</v>
       </c>
@@ -34974,7 +34991,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="192" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" ht="192" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>220</v>
       </c>
@@ -35021,7 +35038,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="30" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" ht="30" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>220</v>
       </c>
@@ -35051,7 +35068,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="45" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" ht="45" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>220</v>
       </c>
@@ -35098,7 +35115,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="60" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" ht="60" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>220</v>
       </c>
@@ -35201,7 +35218,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="49" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A49" s="33" t="s">
         <v>168</v>
       </c>
@@ -35240,7 +35257,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="50" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A50" s="33" t="s">
         <v>170</v>
       </c>
@@ -35279,7 +35296,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="51" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A51" s="33" t="s">
         <v>172</v>
       </c>
@@ -35318,7 +35335,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="52" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A52" s="33" t="s">
         <v>174</v>
       </c>
@@ -35357,7 +35374,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="53" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A53" s="33" t="s">
         <v>176</v>
       </c>
@@ -35396,7 +35413,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="54" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A54" s="33" t="s">
         <v>178</v>
       </c>
@@ -35435,7 +35452,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="55" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A55" s="33" t="s">
         <v>180</v>
       </c>
@@ -35474,7 +35491,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="56" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A56" s="33" t="s">
         <v>182</v>
       </c>
@@ -35513,7 +35530,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="57" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A57" s="33" t="s">
         <v>184</v>
       </c>
@@ -35552,7 +35569,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="58" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A58" s="33" t="s">
         <v>235</v>
       </c>
@@ -35591,7 +35608,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="59" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A59" s="33" t="s">
         <v>238</v>
       </c>
@@ -35630,7 +35647,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="60" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A60" s="33" t="s">
         <v>240</v>
       </c>
@@ -35669,7 +35686,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="61" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A61" s="33" t="s">
         <v>242</v>
       </c>
@@ -35708,7 +35725,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="62" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A62" s="33" t="s">
         <v>245</v>
       </c>
@@ -35747,7 +35764,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="63" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A63" s="33" t="s">
         <v>247</v>
       </c>
@@ -35786,7 +35803,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="64" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A64" s="33" t="s">
         <v>249</v>
       </c>
@@ -35825,7 +35842,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="65" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A65" s="33" t="s">
         <v>251</v>
       </c>
@@ -35864,7 +35881,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="66" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A66" s="33" t="s">
         <v>253</v>
       </c>
@@ -35903,7 +35920,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="33" t="s">
         <v>255</v>
       </c>
@@ -35942,7 +35959,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="68" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A68" s="33" t="s">
         <v>257</v>
       </c>
@@ -35981,7 +35998,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="69" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A69" s="33" t="s">
         <v>259</v>
       </c>
@@ -36020,7 +36037,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="70" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A70" s="33" t="s">
         <v>261</v>
       </c>
@@ -36059,7 +36076,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="71" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A71" s="33" t="s">
         <v>263</v>
       </c>
@@ -36098,7 +36115,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="72" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A72" s="33" t="s">
         <v>265</v>
       </c>
@@ -36137,7 +36154,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="73" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A73" s="33" t="s">
         <v>267</v>
       </c>
@@ -36176,7 +36193,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="74" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A74" s="33" t="s">
         <v>269</v>
       </c>
@@ -36215,7 +36232,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="75" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A75" s="33" t="s">
         <v>271</v>
       </c>
@@ -36254,7 +36271,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="76" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A76" s="33" t="s">
         <v>273</v>
       </c>
@@ -36293,7 +36310,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="77" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A77" s="33" t="s">
         <v>275</v>
       </c>
@@ -36332,7 +36349,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="78" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A78" s="33" t="s">
         <v>277</v>
       </c>
@@ -36371,7 +36388,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="79" spans="1:19" ht="48" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:19" ht="48" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="33" t="s">
         <v>279</v>
       </c>
@@ -36410,7 +36427,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="80" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A80" s="33" t="s">
         <v>281</v>
       </c>
@@ -36449,7 +36466,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="81" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A81" s="33" t="s">
         <v>283</v>
       </c>
@@ -36488,7 +36505,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="82" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="33" t="s">
         <v>285</v>
       </c>
@@ -36527,7 +36544,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A83" s="33" t="s">
         <v>287</v>
       </c>
@@ -36566,7 +36583,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A84" s="33" t="s">
         <v>289</v>
       </c>
@@ -36605,7 +36622,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A85" s="33" t="s">
         <v>291</v>
       </c>
@@ -36644,7 +36661,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A86" s="33" t="s">
         <v>293</v>
       </c>
@@ -36683,7 +36700,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A87" s="33" t="s">
         <v>295</v>
       </c>
@@ -36722,7 +36739,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A88" s="33" t="s">
         <v>297</v>
       </c>
@@ -36761,7 +36778,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="89" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="33" t="s">
         <v>302</v>
       </c>
@@ -36800,7 +36817,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="90" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="33" t="s">
         <v>304</v>
       </c>
@@ -36839,7 +36856,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="91" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A91" s="33" t="s">
         <v>306</v>
       </c>
@@ -36878,7 +36895,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="92" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A92" s="33" t="s">
         <v>308</v>
       </c>
@@ -36917,7 +36934,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="93" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A93" s="33" t="s">
         <v>310</v>
       </c>
@@ -37012,7 +37029,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="95" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A95" s="33" t="s">
         <v>360</v>
       </c>
@@ -37051,7 +37068,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="96" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A96" s="33" t="s">
         <v>362</v>
       </c>
@@ -37090,7 +37107,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="97" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A97" s="33" t="s">
         <v>364</v>
       </c>
@@ -37129,7 +37146,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="98" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A98" s="33" t="s">
         <v>366</v>
       </c>
@@ -37168,7 +37185,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A99" s="33" t="s">
         <v>368</v>
       </c>
@@ -37207,7 +37224,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="100" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A100" s="33" t="s">
         <v>370</v>
       </c>
@@ -37246,7 +37263,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="101" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A101" s="33" t="s">
         <v>372</v>
       </c>
@@ -37285,7 +37302,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A102" s="33" t="s">
         <v>374</v>
       </c>
@@ -37324,7 +37341,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A103" s="33" t="s">
         <v>376</v>
       </c>
@@ -37363,7 +37380,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="104" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A104" s="33" t="s">
         <v>378</v>
       </c>
@@ -37402,7 +37419,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A105" s="33" t="s">
         <v>380</v>
       </c>
@@ -37441,7 +37458,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="106" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A106" s="33" t="s">
         <v>382</v>
       </c>
@@ -37480,7 +37497,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="107" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A107" s="33" t="s">
         <v>384</v>
       </c>
@@ -37519,7 +37536,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A108" s="33" t="s">
         <v>386</v>
       </c>
@@ -37558,7 +37575,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A109" s="33" t="s">
         <v>388</v>
       </c>
@@ -37597,7 +37614,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="110" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A110" s="33" t="s">
         <v>390</v>
       </c>
@@ -37636,7 +37653,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A111" s="33" t="s">
         <v>392</v>
       </c>
@@ -37674,7 +37691,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A112" s="33" t="s">
         <v>394</v>
       </c>
@@ -37713,7 +37730,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="113" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A113" s="33" t="s">
         <v>396</v>
       </c>
@@ -37752,7 +37769,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="114" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A114" s="33" t="s">
         <v>398</v>
       </c>
@@ -37791,7 +37808,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="115" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A115" s="33" t="s">
         <v>400</v>
       </c>
@@ -37830,7 +37847,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="116" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A116" s="33" t="s">
         <v>402</v>
       </c>
@@ -37869,7 +37886,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="117" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A117" s="33" t="s">
         <v>404</v>
       </c>
@@ -37908,7 +37925,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="118" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A118" s="33" t="s">
         <v>406</v>
       </c>
@@ -37946,7 +37963,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="119" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A119" s="33" t="s">
         <v>408</v>
       </c>
@@ -37985,7 +38002,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="120" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A120" s="33" t="s">
         <v>410</v>
       </c>
@@ -38024,7 +38041,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="121" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A121" s="33" t="s">
         <v>412</v>
       </c>
@@ -38063,7 +38080,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="122" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A122" s="33" t="s">
         <v>414</v>
       </c>
@@ -38102,7 +38119,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="123" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A123" s="33" t="s">
         <v>416</v>
       </c>
@@ -38140,7 +38157,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="124" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A124" s="33" t="s">
         <v>418</v>
       </c>
@@ -39036,7 +39053,7 @@
       <c r="O139" s="28" t="s">
         <v>972</v>
       </c>
-      <c r="R139" s="54" t="s">
+      <c r="R139" s="6" t="s">
         <v>1273</v>
       </c>
       <c r="S139" s="6" t="s">
@@ -39089,7 +39106,7 @@
       <c r="O140" s="28" t="s">
         <v>972</v>
       </c>
-      <c r="R140" s="54" t="s">
+      <c r="R140" s="6" t="s">
         <v>1273</v>
       </c>
       <c r="S140" s="6" t="s">
@@ -39155,7 +39172,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="142" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
         <v>120</v>
       </c>
@@ -39264,7 +39281,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="120" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:23" ht="105" x14ac:dyDescent="0.3">
       <c r="A144" s="6" t="s">
         <v>431</v>
       </c>
@@ -40096,7 +40113,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:23" ht="30" x14ac:dyDescent="0.3">
       <c r="A157" s="6" t="s">
         <v>220</v>
       </c>
@@ -40337,7 +40354,7 @@
         <v>2023</v>
       </c>
       <c r="O161" s="6"/>
-      <c r="R161" s="54" t="s">
+      <c r="R161" s="6" t="s">
         <v>1264</v>
       </c>
       <c r="S161" s="6" t="s">
@@ -40376,7 +40393,7 @@
         <v>2023</v>
       </c>
       <c r="O162" s="6"/>
-      <c r="R162" s="54" t="s">
+      <c r="R162" s="6" t="s">
         <v>1264</v>
       </c>
       <c r="S162" s="6" t="s">
@@ -40415,7 +40432,7 @@
         <v>2023</v>
       </c>
       <c r="O163" s="6"/>
-      <c r="R163" s="54" t="s">
+      <c r="R163" s="6" t="s">
         <v>1264</v>
       </c>
       <c r="S163" s="6" t="s">
@@ -40454,7 +40471,7 @@
         <v>2023</v>
       </c>
       <c r="O164" s="6"/>
-      <c r="R164" s="54" t="s">
+      <c r="R164" s="6" t="s">
         <v>1264</v>
       </c>
       <c r="S164" s="6" t="s">
@@ -40493,7 +40510,7 @@
         <v>2023</v>
       </c>
       <c r="O165" s="6"/>
-      <c r="R165" s="54" t="s">
+      <c r="R165" s="6" t="s">
         <v>1264</v>
       </c>
       <c r="S165" s="6" t="s">
@@ -40532,7 +40549,7 @@
         <v>2023</v>
       </c>
       <c r="O166" s="6"/>
-      <c r="R166" s="54" t="s">
+      <c r="R166" s="6" t="s">
         <v>1264</v>
       </c>
       <c r="S166" s="6" t="s">
@@ -40571,7 +40588,7 @@
         <v>2023</v>
       </c>
       <c r="O167" s="6"/>
-      <c r="R167" s="54" t="s">
+      <c r="R167" s="6" t="s">
         <v>1267</v>
       </c>
       <c r="S167" s="6" t="s">
@@ -40619,7 +40636,7 @@
         <v>2023</v>
       </c>
       <c r="O168" s="6"/>
-      <c r="R168" s="54" t="s">
+      <c r="R168" s="6" t="s">
         <v>1267</v>
       </c>
       <c r="S168" s="6" t="s">
@@ -40667,7 +40684,7 @@
         <v>2023</v>
       </c>
       <c r="O169" s="6"/>
-      <c r="R169" s="54" t="s">
+      <c r="R169" s="6" t="s">
         <v>1267</v>
       </c>
       <c r="S169" s="6" t="s">
@@ -40715,7 +40732,7 @@
         <v>2023</v>
       </c>
       <c r="O170" s="6"/>
-      <c r="R170" s="54" t="s">
+      <c r="R170" s="6" t="s">
         <v>1267</v>
       </c>
       <c r="S170" s="6" t="s">
@@ -40763,7 +40780,7 @@
         <v>2023</v>
       </c>
       <c r="O171" s="6"/>
-      <c r="R171" s="54" t="s">
+      <c r="R171" s="6" t="s">
         <v>1267</v>
       </c>
       <c r="S171" s="6" t="s">
@@ -40811,7 +40828,7 @@
         <v>2023</v>
       </c>
       <c r="O172" s="6"/>
-      <c r="R172" s="54" t="s">
+      <c r="R172" s="6" t="s">
         <v>1267</v>
       </c>
       <c r="S172" s="6" t="s">
@@ -41074,7 +41091,7 @@
         <v>1269</v>
       </c>
     </row>
-    <row r="178" spans="1:20" ht="75" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:20" ht="75" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
         <v>220</v>
       </c>
@@ -41121,7 +41138,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="179" spans="1:20" ht="60" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:20" ht="60" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>220</v>
       </c>
@@ -41168,7 +41185,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="180" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A180" s="33" t="s">
         <v>150</v>
       </c>
@@ -41207,7 +41224,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="181" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A181" s="33" t="s">
         <v>153</v>
       </c>
@@ -41245,7 +41262,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="182" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A182" s="33" t="s">
         <v>155</v>
       </c>
@@ -41283,7 +41300,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="183" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A183" s="33" t="s">
         <v>157</v>
       </c>
@@ -41322,7 +41339,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="184" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A184" s="33" t="s">
         <v>159</v>
       </c>
@@ -41360,7 +41377,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="185" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A185" s="33" t="s">
         <v>162</v>
       </c>
@@ -41398,7 +41415,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="186" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A186" s="33" t="s">
         <v>164</v>
       </c>
@@ -41437,7 +41454,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="187" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A187" s="33" t="s">
         <v>144</v>
       </c>
@@ -41475,7 +41492,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="188" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A188" s="33" t="s">
         <v>166</v>
       </c>
@@ -41513,7 +41530,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="189" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A189" s="33" t="s">
         <v>312</v>
       </c>
@@ -41552,7 +41569,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="190" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A190" s="33" t="s">
         <v>314</v>
       </c>
@@ -41590,7 +41607,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="191" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A191" s="33" t="s">
         <v>316</v>
       </c>
@@ -41628,7 +41645,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="192" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A192" s="33" t="s">
         <v>318</v>
       </c>
@@ -41667,7 +41684,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="193" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A193" s="33" t="s">
         <v>320</v>
       </c>
@@ -41705,7 +41722,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="194" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A194" s="33" t="s">
         <v>322</v>
       </c>
@@ -41743,7 +41760,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="195" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A195" s="33" t="s">
         <v>324</v>
       </c>
@@ -41782,7 +41799,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="196" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A196" s="33" t="s">
         <v>326</v>
       </c>
@@ -41820,7 +41837,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="197" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A197" s="33" t="s">
         <v>328</v>
       </c>
@@ -42150,7 +42167,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A209" s="38" t="s">
         <v>212</v>
       </c>
@@ -42172,7 +42189,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A210" s="38" t="s">
         <v>216</v>
       </c>
@@ -42194,7 +42211,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A211" s="38" t="s">
         <v>214</v>
       </c>
@@ -42216,7 +42233,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A212" s="38" t="s">
         <v>342</v>
       </c>
@@ -42238,7 +42255,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A213" s="38" t="s">
         <v>344</v>
       </c>
@@ -42260,7 +42277,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A214" s="38" t="s">
         <v>340</v>
       </c>
@@ -42282,7 +42299,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A215" s="38" t="s">
         <v>356</v>
       </c>
@@ -42304,7 +42321,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A216" s="38" t="s">
         <v>358</v>
       </c>
@@ -42326,7 +42343,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A217" s="38" t="s">
         <v>354</v>
       </c>
@@ -42348,7 +42365,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A218" s="38" t="s">
         <v>334</v>
       </c>
@@ -42370,7 +42387,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A219" s="38" t="s">
         <v>348</v>
       </c>
@@ -42392,7 +42409,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A220" s="38" t="s">
         <v>336</v>
       </c>
@@ -42414,7 +42431,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A221" s="38" t="s">
         <v>350</v>
       </c>
@@ -42436,15 +42453,52 @@
         <v>41</v>
       </c>
     </row>
+    <row r="222" spans="1:23" ht="90" x14ac:dyDescent="0.3">
+      <c r="F222" s="6" t="s">
+        <v>1299</v>
+      </c>
+      <c r="G222" s="6" t="s">
+        <v>1293</v>
+      </c>
+      <c r="I222" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="J222" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="K222" s="13" t="s">
+        <v>1294</v>
+      </c>
+      <c r="L222" s="13">
+        <v>2024</v>
+      </c>
+      <c r="M222" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="N222" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="O222" s="7" t="s">
+        <v>1298</v>
+      </c>
+      <c r="S222" s="6" t="s">
+        <v>1235</v>
+      </c>
+      <c r="T222" s="10" t="s">
+        <v>1297</v>
+      </c>
+      <c r="U222" s="6" t="s">
+        <v>1295</v>
+      </c>
+      <c r="V222" s="6" t="s">
+        <v>1296</v>
+      </c>
+      <c r="W222" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W221" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}">
-    <filterColumn colId="18">
-      <filters blank="1">
-        <filter val="Completa"/>
-        <filter val="Incompleta"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:W222" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}"/>
   <mergeCells count="1">
     <mergeCell ref="T18:T19"/>
   </mergeCells>
@@ -43885,15 +43939,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="53729c01-e331-46af-8f84-09bea977ed00">
@@ -43906,7 +43951,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EAB170F55A8EC74185BD611F05A04793" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9a7766076c5b4407dfa4a29cb2dc7926">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="53729c01-e331-46af-8f84-09bea977ed00" xmlns:ns3="0b6a0b30-4523-4899-95a0-946babcdb6cb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd836aff7d432d14d0dd9befd298821c" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -44130,15 +44175,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86D2BEE1-3487-46A6-9F52-47008EF3F06B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -44152,7 +44198,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11D6F162-D51B-4B3D-AD62-C00B241D1426}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -44170,4 +44216,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Agrego tablas Vivienda y base para Turismo
</commit_message>
<xml_diff>
--- a/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
+++ b/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAURA\Trabajo\EAFIT\Proyectos\Provincias\git\Proyecto-Provincias\01_Data\00_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40848687-80D0-4615-BF9D-1322E3409D47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9984987C-664F-4748-8695-952D9DBEF71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="5" activeTab="5" xr2:uid="{87AE0CA6-2098-4AEE-924F-4FDC71F02AC8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{87AE0CA6-2098-4AEE-924F-4FDC71F02AC8}"/>
   </bookViews>
   <sheets>
     <sheet name="Diccionario" sheetId="3" r:id="rId1"/>
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Diccionario_Base!$A$1:$I$221</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Distribución homogeneización'!$A$1:$C$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Indicadores adicionales'!$A$1:$C$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Indicadores clave'!$A$1:$W$222</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Indicadores clave'!$A$1:$W$224</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inventario variables'!$A$1:$Q$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Variables nuevas (propuesta)'!$A$1:$J$2</definedName>
   </definedNames>
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8875" uniqueCount="1300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8923" uniqueCount="1319">
   <si>
     <t>Tipo</t>
   </si>
@@ -4081,6 +4081,63 @@
   </si>
   <si>
     <t xml:space="preserve">Tasa de mortalidad general por cada cien mil habitantes </t>
+  </si>
+  <si>
+    <t>Índice de riesgo ajustado por capacidades (EXCESO DE LLUVIAS)</t>
+  </si>
+  <si>
+    <t>Índice de riesgo ajustado por capacidades (DÉFICIT DE LLUVIAS)</t>
+  </si>
+  <si>
+    <t>IMRC_E</t>
+  </si>
+  <si>
+    <t>IMRC_D</t>
+  </si>
+  <si>
+    <t>Indice gestion capacidades 2024.xlsx (hoja: Exceso de lluvias)</t>
+  </si>
+  <si>
+    <t>Indice gestion capacidades 2024.xlsx (hoja: Déficit de lluvias)</t>
+  </si>
+  <si>
+    <t>Se agregó Indice gestion capacidades 2024.xlsx, hoja "Exceso de lluvias". Fuente: https://www.dnp.gov.co/LaEntidad_/subdireccion-general-prospectiva-desarrollo-nacional/direccion-ambiente-desarrollo-sostenible/Paginas/indice-municipal-de-gestion-de-riesgo-ajustado-por-capacidades.aspx</t>
+  </si>
+  <si>
+    <t>Se agregó Indice gestion capacidades 2024.xlsx, hoja "Déficit de lluvias". Fuente: https://www.dnp.gov.co/LaEntidad_/subdireccion-general-prospectiva-desarrollo-nacional/direccion-ambiente-desarrollo-sostenible/Paginas/indice-municipal-de-gestion-de-riesgo-ajustado-por-capacidades.aspx</t>
+  </si>
+  <si>
+    <t>Indice gestion capacidades 2024.xlsx, hoja "Exceso de lluvias"</t>
+  </si>
+  <si>
+    <t>Indice gestion capacidades 2024.xlsx, hoja "Déficit de lluvias"</t>
+  </si>
+  <si>
+    <t>Visitantes Extranjeros No residentes</t>
+  </si>
+  <si>
+    <t>conteo_extranjeros</t>
+  </si>
+  <si>
+    <t>Conteo</t>
+  </si>
+  <si>
+    <t>SITA Observatorio de Turismo Sostenible de Antioquia - Gobernación de Antioquia</t>
+  </si>
+  <si>
+    <t>2015-2026</t>
+  </si>
+  <si>
+    <t>2019-2023</t>
+  </si>
+  <si>
+    <t>Turismo.xlsx (hoja: Conteo Extranjeros)</t>
+  </si>
+  <si>
+    <t>Se agregó Turismo.xlsx, hoja "Conteo Extranjeros". Fuente: https://secretaria.turismoantioquia.travel/cifras-turisticas-regionales/</t>
+  </si>
+  <si>
+    <t>SITA_BD (VENR) - Actualizado Enero 2026.xlsx</t>
   </si>
 </sst>
 </file>
@@ -32787,7 +32844,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}">
-  <dimension ref="A1:W222"/>
+  <dimension ref="A1:W225"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" style="6" bestFit="1" customWidth="1"/>
@@ -32803,7 +32860,7 @@
     <col min="12" max="12" width="13.109375" style="13" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="16.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.44140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="42.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="69.109375" style="7" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="50.44140625" style="31" customWidth="1"/>
     <col min="17" max="17" width="14.21875" style="6" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="108" style="6" bestFit="1" customWidth="1"/>
@@ -42454,6 +42511,15 @@
       </c>
     </row>
     <row r="222" spans="1:23" ht="90" x14ac:dyDescent="0.3">
+      <c r="C222" s="6" t="s">
+        <v>1299</v>
+      </c>
+      <c r="D222" s="6" t="s">
+        <v>1299</v>
+      </c>
+      <c r="E222" s="6" t="s">
+        <v>1299</v>
+      </c>
       <c r="F222" s="6" t="s">
         <v>1299</v>
       </c>
@@ -42497,8 +42563,161 @@
         <v>149</v>
       </c>
     </row>
+    <row r="223" spans="1:23" ht="210" x14ac:dyDescent="0.3">
+      <c r="C223" s="6" t="s">
+        <v>1300</v>
+      </c>
+      <c r="D223" s="6" t="s">
+        <v>1300</v>
+      </c>
+      <c r="E223" s="6" t="s">
+        <v>1300</v>
+      </c>
+      <c r="F223" s="6" t="s">
+        <v>1300</v>
+      </c>
+      <c r="G223" s="6" t="s">
+        <v>1302</v>
+      </c>
+      <c r="I223" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="J223" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="K223" s="13">
+        <v>2024</v>
+      </c>
+      <c r="L223" s="13">
+        <v>2024</v>
+      </c>
+      <c r="M223" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="N223" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="O223" s="7" t="s">
+        <v>1304</v>
+      </c>
+      <c r="S223" s="6" t="s">
+        <v>1235</v>
+      </c>
+      <c r="T223" s="10" t="s">
+        <v>1306</v>
+      </c>
+      <c r="U223" s="6" t="s">
+        <v>1308</v>
+      </c>
+      <c r="W223" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="224" spans="1:23" ht="210" x14ac:dyDescent="0.3">
+      <c r="C224" s="6" t="s">
+        <v>1301</v>
+      </c>
+      <c r="D224" s="6" t="s">
+        <v>1301</v>
+      </c>
+      <c r="E224" s="6" t="s">
+        <v>1301</v>
+      </c>
+      <c r="F224" s="6" t="s">
+        <v>1301</v>
+      </c>
+      <c r="G224" s="6" t="s">
+        <v>1303</v>
+      </c>
+      <c r="I224" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="J224" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="K224" s="13">
+        <v>2024</v>
+      </c>
+      <c r="L224" s="13">
+        <v>2024</v>
+      </c>
+      <c r="M224" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="N224" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="O224" s="7" t="s">
+        <v>1305</v>
+      </c>
+      <c r="S224" s="6" t="s">
+        <v>1235</v>
+      </c>
+      <c r="T224" s="10" t="s">
+        <v>1307</v>
+      </c>
+      <c r="U224" s="6" t="s">
+        <v>1309</v>
+      </c>
+      <c r="W224" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="225" spans="3:23" ht="90" x14ac:dyDescent="0.3">
+      <c r="C225" s="6" t="s">
+        <v>1310</v>
+      </c>
+      <c r="D225" s="6" t="s">
+        <v>1310</v>
+      </c>
+      <c r="E225" s="6" t="s">
+        <v>1310</v>
+      </c>
+      <c r="F225" s="6" t="s">
+        <v>1310</v>
+      </c>
+      <c r="G225" s="6" t="s">
+        <v>1311</v>
+      </c>
+      <c r="I225" s="6" t="s">
+        <v>1312</v>
+      </c>
+      <c r="J225" s="6" t="s">
+        <v>1313</v>
+      </c>
+      <c r="K225" s="13" t="s">
+        <v>1314</v>
+      </c>
+      <c r="L225" s="13" t="s">
+        <v>1315</v>
+      </c>
+      <c r="M225" s="6" t="s">
+        <v>894</v>
+      </c>
+      <c r="N225" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="O225" s="7" t="s">
+        <v>1316</v>
+      </c>
+      <c r="S225" s="6" t="s">
+        <v>1235</v>
+      </c>
+      <c r="T225" s="10" t="s">
+        <v>1317</v>
+      </c>
+      <c r="U225" s="6" t="s">
+        <v>1316</v>
+      </c>
+      <c r="V225" s="6" t="s">
+        <v>1318</v>
+      </c>
+      <c r="W225" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W222" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}"/>
+  <autoFilter ref="A1:W224" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}"/>
   <mergeCells count="1">
     <mergeCell ref="T18:T19"/>
   </mergeCells>
@@ -43939,6 +44158,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="53729c01-e331-46af-8f84-09bea977ed00">
@@ -43951,7 +44179,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100EAB170F55A8EC74185BD611F05A04793" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9a7766076c5b4407dfa4a29cb2dc7926">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="53729c01-e331-46af-8f84-09bea977ed00" xmlns:ns3="0b6a0b30-4523-4899-95a0-946babcdb6cb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd836aff7d432d14d0dd9befd298821c" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -44175,16 +44403,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86D2BEE1-3487-46A6-9F52-47008EF3F06B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -44198,7 +44425,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11D6F162-D51B-4B3D-AD62-C00B241D1426}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -44216,12 +44443,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Subo tablas de seguridad
</commit_message>
<xml_diff>
--- a/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
+++ b/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAURA\Trabajo\EAFIT\Proyectos\Provincias\git\Proyecto-Provincias\01_Data\00_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2757037-C15A-411B-A7BC-48421B8C9F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AFE8AFC-A286-4C13-9B1A-1CE78DCBE28D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{87AE0CA6-2098-4AEE-924F-4FDC71F02AC8}"/>
   </bookViews>
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8933" uniqueCount="1325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8934" uniqueCount="1326">
   <si>
     <t>Tipo</t>
   </si>
@@ -4156,6 +4156,9 @@
   </si>
   <si>
     <t>Transporte</t>
+  </si>
+  <si>
+    <t>LLENAR SEGURIDAD (POLICIA Y VICTIMAS)</t>
   </si>
 </sst>
 </file>
@@ -32862,7 +32865,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}">
-  <dimension ref="A1:W230"/>
+  <dimension ref="A1:W231"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" style="6" bestFit="1" customWidth="1"/>
@@ -42772,6 +42775,11 @@
       </c>
       <c r="J230" s="6" t="s">
         <v>1319</v>
+      </c>
+    </row>
+    <row r="231" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="J231" s="6" t="s">
+        <v>1325</v>
       </c>
     </row>
   </sheetData>
@@ -44440,6 +44448,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="53729c01-e331-46af-8f84-09bea977ed00">
@@ -44450,15 +44467,6 @@
     <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -44482,6 +44490,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86D2BEE1-3487-46A6-9F52-47008EF3F06B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -44493,12 +44509,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Agrego archivos faltantes de gobernanza, seguridad, CTI, etc.
</commit_message>
<xml_diff>
--- a/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
+++ b/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAURA\Trabajo\EAFIT\Proyectos\Provincias\git\Proyecto-Provincias\01_Data\00_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AFE8AFC-A286-4C13-9B1A-1CE78DCBE28D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B5F9E7-6CA1-4FD7-AF80-8E75B776A4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{87AE0CA6-2098-4AEE-924F-4FDC71F02AC8}"/>
   </bookViews>
@@ -32,7 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Inventario variables'!$A$1:$Q$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Variables nuevas (propuesta)'!$A$1:$J$2</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId10"/>
   </pivotCaches>
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8934" uniqueCount="1326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8938" uniqueCount="1330">
   <si>
     <t>Tipo</t>
   </si>
@@ -4159,6 +4159,18 @@
   </si>
   <si>
     <t>LLENAR SEGURIDAD (POLICIA Y VICTIMAS)</t>
+  </si>
+  <si>
+    <t>LLENAR VARIABLES DE ENERGÍA</t>
+  </si>
+  <si>
+    <t>LLENAR VARIABLES DE GOBERNANZA Y PAZ</t>
+  </si>
+  <si>
+    <t>LLENAR INTERNET FIJO, ÍNDICE DE GOBERNANZA DIGITAL</t>
+  </si>
+  <si>
+    <t>VARIABLES DE PAZ</t>
   </si>
 </sst>
 </file>
@@ -32865,7 +32877,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}">
-  <dimension ref="A1:W231"/>
+  <dimension ref="A1:W235"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" style="6" bestFit="1" customWidth="1"/>
@@ -42780,6 +42792,26 @@
     <row r="231" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J231" s="6" t="s">
         <v>1325</v>
+      </c>
+    </row>
+    <row r="232" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="J232" s="6" t="s">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="233" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="J233" s="6" t="s">
+        <v>1327</v>
+      </c>
+    </row>
+    <row r="234" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="J234" s="6" t="s">
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="235" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="J235" s="6" t="s">
+        <v>1329</v>
       </c>
     </row>
   </sheetData>
@@ -44448,15 +44480,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="53729c01-e331-46af-8f84-09bea977ed00">
@@ -44467,6 +44490,15 @@
     <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -44490,14 +44522,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86D2BEE1-3487-46A6-9F52-47008EF3F06B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -44509,4 +44533,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C347E16F-80D6-4386-AB0F-BCEE924F2FE1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualización integral del pipeline: suicidios 2022-2024, reparación colectiva UARIV, ingresos de inversión, resumen-viñeta y correcciones de Pablo
Incorpora las 20 correcciones reportadas por Pablo (pandoc/RSTUDIO_PANDOC entre otras),
suma nuevas fuentes (DANE Cuadro 15 + SIVIGILA por residencia para suicidios/intentos
2022-2024, sujetos de reparación colectiva UARIV, ingresos de inversión por fuente vía
API de Mapa de Inversiones DNP) y agrega un resumen-viñeta por dimensión en los informes.
Corre limpio para las 11 provincias más el comparativo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
+++ b/01_Data/00_Inputs/INVENTARIO_VARIABLES_v_2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAURA\Trabajo\EAFIT\Proyectos\Provincias\git\Proyecto-Provincias\01_Data\00_Inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\LAURA\Trabajo\EAFIT\Proyectos\Provincias\git\Proyecto-Provincias-nuevo\01_Data\00_Inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B5F9E7-6CA1-4FD7-AF80-8E75B776A4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D90A03D-0278-4EB9-BACB-0E15B66487E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{87AE0CA6-2098-4AEE-924F-4FDC71F02AC8}"/>
   </bookViews>
@@ -166,7 +166,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8938" uniqueCount="1330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8951" uniqueCount="1332">
   <si>
     <t>Tipo</t>
   </si>
@@ -4059,9 +4059,6 @@
     <t>Se actualizó DATOS SALUD.xlsx, hoja "desnutri_aguda&lt;5 tasax100mil&lt;5". Fuente: https://dssa.gov.co/OSSSA/Vigilancia%20en%20Salud%20P%C3%BAblica.html</t>
   </si>
   <si>
-    <t>Sí está en la base de datos, pero no consigo la información</t>
-  </si>
-  <si>
     <t>tasa_mortalidad</t>
   </si>
   <si>
@@ -4171,6 +4168,15 @@
   </si>
   <si>
     <t>VARIABLES DE PAZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se agreggó a INPUTS el dato de 2024 (disponible 2025, pero por homogeneización se deja ese año). Disponible en: https://portalsivigila.ins.gov.co/Paginas/Buscador.aspx# </t>
+  </si>
+  <si>
+    <t>Esta variable se construye luego ponderando por población. Pero el dato de intento de suicidio crudo está en SIVIGILA</t>
+  </si>
+  <si>
+    <t>SUJETOS COLECTIVOS VÍCTIMAS: https://vgv.unidadvictimas.gov.co/sujetos/</t>
   </si>
 </sst>
 </file>
@@ -32877,7 +32883,8 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}">
-  <dimension ref="A1:W235"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:W236"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" style="6" bestFit="1" customWidth="1"/>
@@ -32976,7 +32983,7 @@
         <v>1268</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="60" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
         <v>221</v>
       </c>
@@ -33037,7 +33044,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="150" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" ht="150" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="33" t="s">
         <v>225</v>
       </c>
@@ -33095,7 +33102,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="165" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" ht="165" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="33" t="s">
         <v>227</v>
       </c>
@@ -33157,7 +33164,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" ht="55.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="33" t="s">
         <v>229</v>
       </c>
@@ -33215,7 +33222,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>124</v>
       </c>
@@ -33271,7 +33278,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>424</v>
       </c>
@@ -33327,7 +33334,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>426</v>
       </c>
@@ -33383,7 +33390,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="9" spans="1:23" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" ht="27.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>443</v>
       </c>
@@ -33440,7 +33447,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="10" spans="1:23" ht="79.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" ht="79.8" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>457</v>
       </c>
@@ -33497,7 +33504,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="11" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>220</v>
       </c>
@@ -33544,7 +33551,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>220</v>
       </c>
@@ -33588,7 +33595,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="13" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>220</v>
       </c>
@@ -33624,7 +33631,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>112</v>
       </c>
@@ -33677,7 +33684,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" ht="23.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>220</v>
       </c>
@@ -33721,7 +33728,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" ht="42.6" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>220</v>
       </c>
@@ -33765,7 +33772,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="17" spans="1:23" ht="31.8" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" ht="31.8" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="33" t="s">
         <v>116</v>
       </c>
@@ -33801,7 +33808,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:23" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="33" t="s">
         <v>186</v>
       </c>
@@ -33863,7 +33870,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:23" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="33" t="s">
         <v>231</v>
       </c>
@@ -33915,7 +33922,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" ht="28.5" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>220</v>
       </c>
@@ -33957,7 +33964,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="21" spans="1:23" ht="104.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" ht="104.25" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>220</v>
       </c>
@@ -33999,7 +34006,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="22" spans="1:23" ht="108.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" ht="108.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>220</v>
       </c>
@@ -34041,7 +34048,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
         <v>220</v>
       </c>
@@ -34083,7 +34090,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
         <v>220</v>
       </c>
@@ -34116,7 +34123,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" ht="45" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>220</v>
       </c>
@@ -34152,7 +34159,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="6" t="s">
         <v>52</v>
       </c>
@@ -34208,7 +34215,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" ht="45" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
         <v>69</v>
       </c>
@@ -34270,7 +34277,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
         <v>72</v>
       </c>
@@ -34332,7 +34339,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="33" t="s">
         <v>76</v>
       </c>
@@ -34378,7 +34385,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" s="33" t="s">
         <v>80</v>
       </c>
@@ -34424,7 +34431,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="33" t="s">
         <v>82</v>
       </c>
@@ -34470,7 +34477,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="33" t="s">
         <v>84</v>
       </c>
@@ -34516,7 +34523,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="6" t="s">
         <v>218</v>
       </c>
@@ -34573,7 +34580,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="30" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="33" t="s">
         <v>299</v>
       </c>
@@ -34618,7 +34625,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="30" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>476</v>
       </c>
@@ -34675,7 +34682,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="36" spans="1:20" ht="30" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
         <v>492</v>
       </c>
@@ -34732,7 +34739,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="30" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="6" t="s">
         <v>506</v>
       </c>
@@ -34789,7 +34796,7 @@
         <v>1245</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="33" t="s">
         <v>508</v>
       </c>
@@ -34834,7 +34841,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33" t="s">
         <v>510</v>
       </c>
@@ -34879,7 +34886,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="33" t="s">
         <v>512</v>
       </c>
@@ -34924,7 +34931,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="33" t="s">
         <v>514</v>
       </c>
@@ -34969,7 +34976,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="6" t="s">
         <v>134</v>
       </c>
@@ -35025,7 +35032,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
         <v>139</v>
       </c>
@@ -35081,7 +35088,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="192" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" ht="192" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
         <v>220</v>
       </c>
@@ -35128,7 +35135,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="30" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>220</v>
       </c>
@@ -35158,7 +35165,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="45" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" ht="45" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
         <v>220</v>
       </c>
@@ -35205,7 +35212,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="60" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" ht="60" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
         <v>220</v>
       </c>
@@ -35252,7 +35259,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
         <v>141</v>
       </c>
@@ -35308,7 +35315,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="33" t="s">
         <v>168</v>
       </c>
@@ -35347,7 +35354,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" s="33" t="s">
         <v>170</v>
       </c>
@@ -35386,7 +35393,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" s="33" t="s">
         <v>172</v>
       </c>
@@ -35425,7 +35432,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="33" t="s">
         <v>174</v>
       </c>
@@ -35464,7 +35471,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" s="33" t="s">
         <v>176</v>
       </c>
@@ -35503,7 +35510,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="33" t="s">
         <v>178</v>
       </c>
@@ -35542,7 +35549,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="33" t="s">
         <v>180</v>
       </c>
@@ -35581,7 +35588,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="33" t="s">
         <v>182</v>
       </c>
@@ -35620,7 +35627,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="33" t="s">
         <v>184</v>
       </c>
@@ -35659,7 +35666,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="33" t="s">
         <v>235</v>
       </c>
@@ -35698,7 +35705,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="33" t="s">
         <v>238</v>
       </c>
@@ -35737,7 +35744,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="33" t="s">
         <v>240</v>
       </c>
@@ -35776,7 +35783,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="33" t="s">
         <v>242</v>
       </c>
@@ -35815,7 +35822,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="33" t="s">
         <v>245</v>
       </c>
@@ -35854,7 +35861,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" s="33" t="s">
         <v>247</v>
       </c>
@@ -35893,7 +35900,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="33" t="s">
         <v>249</v>
       </c>
@@ -35932,7 +35939,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="33" t="s">
         <v>251</v>
       </c>
@@ -35971,7 +35978,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="33" t="s">
         <v>253</v>
       </c>
@@ -36010,7 +36017,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="67" spans="1:19" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:19" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="33" t="s">
         <v>255</v>
       </c>
@@ -36049,7 +36056,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="33" t="s">
         <v>257</v>
       </c>
@@ -36088,7 +36095,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="33" t="s">
         <v>259</v>
       </c>
@@ -36127,7 +36134,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" s="33" t="s">
         <v>261</v>
       </c>
@@ -36166,7 +36173,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="33" t="s">
         <v>263</v>
       </c>
@@ -36205,7 +36212,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="33" t="s">
         <v>265</v>
       </c>
@@ -36244,7 +36251,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="33" t="s">
         <v>267</v>
       </c>
@@ -36283,7 +36290,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="33" t="s">
         <v>269</v>
       </c>
@@ -36322,7 +36329,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="33" t="s">
         <v>271</v>
       </c>
@@ -36361,7 +36368,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="33" t="s">
         <v>273</v>
       </c>
@@ -36400,7 +36407,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77" s="33" t="s">
         <v>275</v>
       </c>
@@ -36439,7 +36446,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="33" t="s">
         <v>277</v>
       </c>
@@ -36478,7 +36485,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="79" spans="1:19" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:19" ht="48" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="33" t="s">
         <v>279</v>
       </c>
@@ -36517,7 +36524,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="80" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80" s="33" t="s">
         <v>281</v>
       </c>
@@ -36556,7 +36563,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="33" t="s">
         <v>283</v>
       </c>
@@ -36595,7 +36602,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="82" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="33" t="s">
         <v>285</v>
       </c>
@@ -36634,7 +36641,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="33" t="s">
         <v>287</v>
       </c>
@@ -36673,7 +36680,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="33" t="s">
         <v>289</v>
       </c>
@@ -36712,7 +36719,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="33" t="s">
         <v>291</v>
       </c>
@@ -36751,7 +36758,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="33" t="s">
         <v>293</v>
       </c>
@@ -36790,7 +36797,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="33" t="s">
         <v>295</v>
       </c>
@@ -36829,7 +36836,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88" s="33" t="s">
         <v>297</v>
       </c>
@@ -36868,7 +36875,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="89" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="33" t="s">
         <v>302</v>
       </c>
@@ -36907,7 +36914,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="90" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="33" t="s">
         <v>304</v>
       </c>
@@ -36946,7 +36953,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="33" t="s">
         <v>306</v>
       </c>
@@ -36985,7 +36992,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="33" t="s">
         <v>308</v>
       </c>
@@ -37024,7 +37031,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="33" t="s">
         <v>310</v>
       </c>
@@ -37063,7 +37070,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94" s="6" t="s">
         <v>330</v>
       </c>
@@ -37119,7 +37126,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="33" t="s">
         <v>360</v>
       </c>
@@ -37158,7 +37165,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="33" t="s">
         <v>362</v>
       </c>
@@ -37197,7 +37204,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="97" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="33" t="s">
         <v>364</v>
       </c>
@@ -37236,7 +37243,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="98" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="33" t="s">
         <v>366</v>
       </c>
@@ -37275,7 +37282,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="99" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="33" t="s">
         <v>368</v>
       </c>
@@ -37314,7 +37321,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="100" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="33" t="s">
         <v>370</v>
       </c>
@@ -37353,7 +37360,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="101" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="33" t="s">
         <v>372</v>
       </c>
@@ -37392,7 +37399,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="102" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="33" t="s">
         <v>374</v>
       </c>
@@ -37431,7 +37438,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="103" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="33" t="s">
         <v>376</v>
       </c>
@@ -37470,7 +37477,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="104" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="33" t="s">
         <v>378</v>
       </c>
@@ -37509,7 +37516,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="105" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="33" t="s">
         <v>380</v>
       </c>
@@ -37548,7 +37555,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="106" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" s="33" t="s">
         <v>382</v>
       </c>
@@ -37587,7 +37594,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="107" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" s="33" t="s">
         <v>384</v>
       </c>
@@ -37626,7 +37633,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="108" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="33" t="s">
         <v>386</v>
       </c>
@@ -37665,7 +37672,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="109" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="33" t="s">
         <v>388</v>
       </c>
@@ -37704,7 +37711,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="110" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="33" t="s">
         <v>390</v>
       </c>
@@ -37743,7 +37750,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="111" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="33" t="s">
         <v>392</v>
       </c>
@@ -37781,7 +37788,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="112" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:19" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" s="33" t="s">
         <v>394</v>
       </c>
@@ -37820,7 +37827,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="33" t="s">
         <v>396</v>
       </c>
@@ -37859,7 +37866,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="33" t="s">
         <v>398</v>
       </c>
@@ -37898,7 +37905,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="33" t="s">
         <v>400</v>
       </c>
@@ -37937,7 +37944,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="33" t="s">
         <v>402</v>
       </c>
@@ -37976,7 +37983,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="33" t="s">
         <v>404</v>
       </c>
@@ -38015,7 +38022,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="33" t="s">
         <v>406</v>
       </c>
@@ -38053,7 +38060,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="33" t="s">
         <v>408</v>
       </c>
@@ -38092,7 +38099,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="33" t="s">
         <v>410</v>
       </c>
@@ -38131,7 +38138,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="121" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="33" t="s">
         <v>412</v>
       </c>
@@ -38170,7 +38177,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="122" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="33" t="s">
         <v>414</v>
       </c>
@@ -38209,7 +38216,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="33" t="s">
         <v>416</v>
       </c>
@@ -38247,7 +38254,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="33" t="s">
         <v>418</v>
       </c>
@@ -38286,7 +38293,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="35" t="s">
         <v>428</v>
       </c>
@@ -38348,7 +38355,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="75" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:23" ht="75" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" s="6" t="s">
         <v>220</v>
       </c>
@@ -38401,7 +38408,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="127" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:23" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="6" t="s">
         <v>220</v>
       </c>
@@ -38454,7 +38461,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="75" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:23" ht="75" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="6" t="s">
         <v>220</v>
       </c>
@@ -38507,7 +38514,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="120" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:23" ht="120" hidden="1" x14ac:dyDescent="0.3">
       <c r="A129" s="6" t="s">
         <v>220</v>
       </c>
@@ -38557,7 +38564,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="90" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:23" ht="90" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="6" t="s">
         <v>220</v>
       </c>
@@ -38610,7 +38617,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="75" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:23" ht="75" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="6" t="s">
         <v>220</v>
       </c>
@@ -38663,7 +38670,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="132" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="6" t="s">
         <v>437</v>
       </c>
@@ -38732,7 +38739,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="133" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="6" t="s">
         <v>441</v>
       </c>
@@ -38801,7 +38808,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="134" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="6" t="s">
         <v>451</v>
       </c>
@@ -38861,7 +38868,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="6" t="s">
         <v>455</v>
       </c>
@@ -38921,7 +38928,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="6" t="s">
         <v>480</v>
       </c>
@@ -38990,7 +38997,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" s="6" t="s">
         <v>484</v>
       </c>
@@ -39062,7 +39069,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="6" t="s">
         <v>220</v>
       </c>
@@ -39109,7 +39116,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="90" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:23" ht="90" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="6" t="s">
         <v>220</v>
       </c>
@@ -39162,7 +39169,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="90" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:23" ht="90" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="6" t="s">
         <v>220</v>
       </c>
@@ -39215,7 +39222,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="6" t="s">
         <v>220</v>
       </c>
@@ -39262,7 +39269,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" s="6" t="s">
         <v>120</v>
       </c>
@@ -39315,7 +39322,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="143" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" s="6" t="s">
         <v>233</v>
       </c>
@@ -39371,7 +39378,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="105" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:23" ht="105" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="6" t="s">
         <v>431</v>
       </c>
@@ -39443,7 +39450,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="6" t="s">
         <v>434</v>
       </c>
@@ -39512,7 +39519,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="6" t="s">
         <v>439</v>
       </c>
@@ -39581,7 +39588,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="147" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:23" ht="45" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="6" t="s">
         <v>449</v>
       </c>
@@ -39641,7 +39648,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:23" ht="45" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="6" t="s">
         <v>453</v>
       </c>
@@ -39701,7 +39708,7 @@
         <v>1290</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="6" t="s">
         <v>478</v>
       </c>
@@ -39770,7 +39777,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="6" t="s">
         <v>482</v>
       </c>
@@ -39839,7 +39846,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="135" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:23" ht="135" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" s="6" t="s">
         <v>501</v>
       </c>
@@ -39908,7 +39915,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="90" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:23" ht="90" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="6" t="s">
         <v>199</v>
       </c>
@@ -39967,7 +39974,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="153" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A153" s="6" t="s">
         <v>332</v>
       </c>
@@ -40026,7 +40033,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="154" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="6" t="s">
         <v>338</v>
       </c>
@@ -40085,7 +40092,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="155" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="6" t="s">
         <v>346</v>
       </c>
@@ -40144,7 +40151,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="6" t="s">
         <v>352</v>
       </c>
@@ -40203,7 +40210,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="30" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:23" ht="30" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="6" t="s">
         <v>220</v>
       </c>
@@ -40247,7 +40254,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="120" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:23" ht="120" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="6" t="s">
         <v>220</v>
       </c>
@@ -40303,7 +40310,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="120" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:23" ht="120" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="6" t="s">
         <v>220</v>
       </c>
@@ -40359,7 +40366,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="120" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:23" ht="120" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="6" t="s">
         <v>220</v>
       </c>
@@ -40415,7 +40422,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="161" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:23" ht="135" x14ac:dyDescent="0.3">
       <c r="A161" s="33" t="s">
         <v>191</v>
       </c>
@@ -40448,10 +40455,16 @@
         <v>1264</v>
       </c>
       <c r="S161" s="6" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="T161" s="10" t="s">
-        <v>1292</v>
+        <v>1329</v>
+      </c>
+      <c r="U161" s="6" t="s">
+        <v>1330</v>
+      </c>
+      <c r="W161" s="6" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="162" spans="1:23" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -40487,13 +40500,19 @@
         <v>1264</v>
       </c>
       <c r="S162" s="6" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="T162" s="10" t="s">
-        <v>1292</v>
-      </c>
-    </row>
-    <row r="163" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+        <v>1329</v>
+      </c>
+      <c r="U162" s="6" t="s">
+        <v>1330</v>
+      </c>
+      <c r="W162" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="163" spans="1:23" ht="135" x14ac:dyDescent="0.3">
       <c r="A163" s="33" t="s">
         <v>197</v>
       </c>
@@ -40526,13 +40545,19 @@
         <v>1264</v>
       </c>
       <c r="S163" s="6" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="T163" s="10" t="s">
-        <v>1292</v>
-      </c>
-    </row>
-    <row r="164" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+        <v>1329</v>
+      </c>
+      <c r="U163" s="6" t="s">
+        <v>1330</v>
+      </c>
+      <c r="W163" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="164" spans="1:23" ht="135" x14ac:dyDescent="0.3">
       <c r="A164" s="33" t="s">
         <v>463</v>
       </c>
@@ -40565,13 +40590,19 @@
         <v>1264</v>
       </c>
       <c r="S164" s="6" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="T164" s="10" t="s">
-        <v>1292</v>
-      </c>
-    </row>
-    <row r="165" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+        <v>1329</v>
+      </c>
+      <c r="U164" s="6" t="s">
+        <v>1330</v>
+      </c>
+      <c r="W164" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="165" spans="1:23" ht="135" x14ac:dyDescent="0.3">
       <c r="A165" s="33" t="s">
         <v>465</v>
       </c>
@@ -40604,10 +40635,16 @@
         <v>1264</v>
       </c>
       <c r="S165" s="6" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="T165" s="10" t="s">
-        <v>1292</v>
+        <v>1329</v>
+      </c>
+      <c r="U165" s="6" t="s">
+        <v>1330</v>
+      </c>
+      <c r="W165" s="6" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="166" spans="1:23" ht="15.9" customHeight="1" x14ac:dyDescent="0.3">
@@ -40643,10 +40680,16 @@
         <v>1264</v>
       </c>
       <c r="S166" s="6" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="T166" s="10" t="s">
-        <v>1292</v>
+        <v>1329</v>
+      </c>
+      <c r="U166" s="6" t="s">
+        <v>1330</v>
+      </c>
+      <c r="W166" s="6" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="167" spans="1:23" ht="210" x14ac:dyDescent="0.3">
@@ -40937,7 +40980,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="173" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="6" t="s">
         <v>220</v>
       </c>
@@ -40984,7 +41027,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="45" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:23" ht="45" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="6" t="s">
         <v>220</v>
       </c>
@@ -41031,7 +41074,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="195" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:23" ht="195" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="6" t="s">
         <v>220</v>
       </c>
@@ -41090,7 +41133,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="176" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:23" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="6" t="s">
         <v>220</v>
       </c>
@@ -41134,7 +41177,7 @@
         <v>1236</v>
       </c>
     </row>
-    <row r="177" spans="1:20" ht="120" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:20" ht="120" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="6" t="s">
         <v>220</v>
       </c>
@@ -41181,7 +41224,7 @@
         <v>1269</v>
       </c>
     </row>
-    <row r="178" spans="1:20" ht="75" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:20" ht="75" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="6" t="s">
         <v>220</v>
       </c>
@@ -41228,7 +41271,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="179" spans="1:20" ht="60" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:20" ht="60" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="6" t="s">
         <v>220</v>
       </c>
@@ -41275,7 +41318,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="180" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="33" t="s">
         <v>150</v>
       </c>
@@ -41314,7 +41357,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="181" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="33" t="s">
         <v>153</v>
       </c>
@@ -41352,7 +41395,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="182" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="33" t="s">
         <v>155</v>
       </c>
@@ -41390,7 +41433,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="183" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="33" t="s">
         <v>157</v>
       </c>
@@ -41429,7 +41472,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="184" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="33" t="s">
         <v>159</v>
       </c>
@@ -41467,7 +41510,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="185" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="33" t="s">
         <v>162</v>
       </c>
@@ -41505,7 +41548,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="186" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="33" t="s">
         <v>164</v>
       </c>
@@ -41544,7 +41587,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="187" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="33" t="s">
         <v>144</v>
       </c>
@@ -41582,7 +41625,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="188" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="33" t="s">
         <v>166</v>
       </c>
@@ -41620,7 +41663,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="189" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="33" t="s">
         <v>312</v>
       </c>
@@ -41659,7 +41702,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="190" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="33" t="s">
         <v>314</v>
       </c>
@@ -41697,7 +41740,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="191" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="33" t="s">
         <v>316</v>
       </c>
@@ -41735,7 +41778,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="192" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="33" t="s">
         <v>318</v>
       </c>
@@ -41774,7 +41817,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="193" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="33" t="s">
         <v>320</v>
       </c>
@@ -41812,7 +41855,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="194" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="33" t="s">
         <v>322</v>
       </c>
@@ -41850,7 +41893,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="195" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="33" t="s">
         <v>324</v>
       </c>
@@ -41889,7 +41932,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="196" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="33" t="s">
         <v>326</v>
       </c>
@@ -41927,7 +41970,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="197" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="33" t="s">
         <v>328</v>
       </c>
@@ -41966,7 +42009,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="198" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:20" ht="15.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>420</v>
       </c>
@@ -42022,7 +42065,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="199" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="6" t="s">
         <v>422</v>
       </c>
@@ -42078,7 +42121,7 @@
         <v>1257</v>
       </c>
     </row>
-    <row r="200" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="6" t="s">
         <v>220</v>
       </c>
@@ -42088,7 +42131,7 @@
       <c r="K200" s="6"/>
       <c r="O200" s="31"/>
     </row>
-    <row r="201" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:20" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="6" t="s">
         <v>220</v>
       </c>
@@ -42101,7 +42144,7 @@
       </c>
       <c r="O201" s="28"/>
     </row>
-    <row r="202" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" s="38" t="s">
         <v>445</v>
       </c>
@@ -42125,7 +42168,7 @@
       </c>
       <c r="O202" s="28"/>
     </row>
-    <row r="203" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" s="38" t="s">
         <v>447</v>
       </c>
@@ -42147,7 +42190,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="204" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" s="38" t="s">
         <v>204</v>
       </c>
@@ -42169,7 +42212,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="205" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" s="38" t="s">
         <v>202</v>
       </c>
@@ -42191,7 +42234,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="206" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" s="38" t="s">
         <v>206</v>
       </c>
@@ -42213,7 +42256,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="207" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="38" t="s">
         <v>210</v>
       </c>
@@ -42235,7 +42278,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="208" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" s="38" t="s">
         <v>208</v>
       </c>
@@ -42257,7 +42300,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="209" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" s="38" t="s">
         <v>212</v>
       </c>
@@ -42279,7 +42322,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="210" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="38" t="s">
         <v>216</v>
       </c>
@@ -42301,7 +42344,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="211" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" s="38" t="s">
         <v>214</v>
       </c>
@@ -42323,7 +42366,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="212" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" s="38" t="s">
         <v>342</v>
       </c>
@@ -42345,7 +42388,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="213" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="38" t="s">
         <v>344</v>
       </c>
@@ -42367,7 +42410,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="214" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="38" t="s">
         <v>340</v>
       </c>
@@ -42389,7 +42432,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="215" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" s="38" t="s">
         <v>356</v>
       </c>
@@ -42411,7 +42454,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="216" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" s="38" t="s">
         <v>358</v>
       </c>
@@ -42433,7 +42476,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="217" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="38" t="s">
         <v>354</v>
       </c>
@@ -42455,7 +42498,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="218" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="38" t="s">
         <v>334</v>
       </c>
@@ -42477,7 +42520,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="219" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" s="38" t="s">
         <v>348</v>
       </c>
@@ -42499,7 +42542,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="220" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="38" t="s">
         <v>336</v>
       </c>
@@ -42521,7 +42564,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="221" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:23" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="38" t="s">
         <v>350</v>
       </c>
@@ -42543,21 +42586,21 @@
         <v>41</v>
       </c>
     </row>
-    <row r="222" spans="1:23" ht="90" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:23" ht="90" hidden="1" x14ac:dyDescent="0.3">
       <c r="C222" s="6" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="D222" s="6" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="E222" s="6" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="F222" s="6" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="G222" s="6" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="I222" s="6" t="s">
         <v>41</v>
@@ -42566,7 +42609,7 @@
         <v>44</v>
       </c>
       <c r="K222" s="13" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="L222" s="13">
         <v>2024</v>
@@ -42578,39 +42621,39 @@
         <v>745</v>
       </c>
       <c r="O222" s="7" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="S222" s="6" t="s">
         <v>1235</v>
       </c>
       <c r="T222" s="10" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="U222" s="6" t="s">
+        <v>1294</v>
+      </c>
+      <c r="V222" s="6" t="s">
         <v>1295</v>
-      </c>
-      <c r="V222" s="6" t="s">
-        <v>1296</v>
       </c>
       <c r="W222" s="6" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="223" spans="1:23" ht="210" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:23" ht="210" hidden="1" x14ac:dyDescent="0.3">
       <c r="C223" s="6" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="D223" s="6" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="E223" s="6" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="F223" s="6" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="G223" s="6" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="I223" s="6" t="s">
         <v>114</v>
@@ -42631,36 +42674,36 @@
         <v>745</v>
       </c>
       <c r="O223" s="7" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="S223" s="6" t="s">
         <v>1235</v>
       </c>
       <c r="T223" s="10" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="U223" s="6" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="W223" s="6" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="224" spans="1:23" ht="210" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:23" ht="210" hidden="1" x14ac:dyDescent="0.3">
       <c r="C224" s="6" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="D224" s="6" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="E224" s="6" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="F224" s="6" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="G224" s="6" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="I224" s="6" t="s">
         <v>114</v>
@@ -42681,16 +42724,16 @@
         <v>745</v>
       </c>
       <c r="O224" s="7" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="S224" s="6" t="s">
         <v>1235</v>
       </c>
       <c r="T224" s="10" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="U224" s="6" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="W224" s="6" t="s">
         <v>149</v>
@@ -42698,31 +42741,31 @@
     </row>
     <row r="225" spans="3:23" ht="90" x14ac:dyDescent="0.3">
       <c r="C225" s="6" t="s">
+        <v>1309</v>
+      </c>
+      <c r="D225" s="6" t="s">
+        <v>1309</v>
+      </c>
+      <c r="E225" s="6" t="s">
+        <v>1309</v>
+      </c>
+      <c r="F225" s="6" t="s">
+        <v>1309</v>
+      </c>
+      <c r="G225" s="6" t="s">
         <v>1310</v>
       </c>
-      <c r="D225" s="6" t="s">
-        <v>1310</v>
-      </c>
-      <c r="E225" s="6" t="s">
-        <v>1310</v>
-      </c>
-      <c r="F225" s="6" t="s">
-        <v>1310</v>
-      </c>
-      <c r="G225" s="6" t="s">
+      <c r="I225" s="6" t="s">
         <v>1311</v>
       </c>
-      <c r="I225" s="6" t="s">
+      <c r="J225" s="6" t="s">
         <v>1312</v>
       </c>
-      <c r="J225" s="6" t="s">
+      <c r="K225" s="13" t="s">
         <v>1313</v>
       </c>
-      <c r="K225" s="13" t="s">
+      <c r="L225" s="13" t="s">
         <v>1314</v>
-      </c>
-      <c r="L225" s="13" t="s">
-        <v>1315</v>
       </c>
       <c r="M225" s="6" t="s">
         <v>894</v>
@@ -42731,19 +42774,19 @@
         <v>745</v>
       </c>
       <c r="O225" s="7" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="S225" s="6" t="s">
         <v>1235</v>
       </c>
       <c r="T225" s="10" t="s">
+        <v>1316</v>
+      </c>
+      <c r="U225" s="6" t="s">
+        <v>1315</v>
+      </c>
+      <c r="V225" s="6" t="s">
         <v>1317</v>
-      </c>
-      <c r="U225" s="6" t="s">
-        <v>1316</v>
-      </c>
-      <c r="V225" s="6" t="s">
-        <v>1318</v>
       </c>
       <c r="W225" s="6" t="s">
         <v>149</v>
@@ -42751,71 +42794,82 @@
     </row>
     <row r="226" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F226" s="6" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="J226" s="6" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="227" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F227" s="6" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="J227" s="6" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="228" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F228" s="6" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="J228" s="6" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="229" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F229" s="6" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="J229" s="6" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="230" spans="3:23" x14ac:dyDescent="0.3">
       <c r="F230" s="6" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="J230" s="6" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="231" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J231" s="6" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="232" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J232" s="6" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="233" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J233" s="6" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="234" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J234" s="6" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="235" spans="3:23" x14ac:dyDescent="0.3">
       <c r="J235" s="6" t="s">
-        <v>1329</v>
+        <v>1328</v>
+      </c>
+    </row>
+    <row r="236" spans="3:23" x14ac:dyDescent="0.3">
+      <c r="J236" s="6" t="s">
+        <v>1331</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W224" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}"/>
+  <autoFilter ref="A1:W224" xr:uid="{5F280BC0-9B68-4877-B035-8C33F0D9A661}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Salud mental"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="T18:T19"/>
   </mergeCells>

</xml_diff>